<commit_message>
Register: Premila Lugstein award free, professional accounting work
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RNuMJNauftwNAHeyi1xsmD
</commit_message>
<xml_diff>
--- a/awards/CTS_Payroll_Setup_Register_21102026.xlsx
+++ b/awards/CTS_Payroll_Setup_Register_21102026.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2104" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2103" uniqueCount="477">
   <si>
     <t xml:space="preserve">CTS Payroll Setup Review: Employee Details Report 21/10/2026</t>
   </si>
@@ -73,7 +73,7 @@
     <t xml:space="preserve">4. Office staff on production agreement</t>
   </si>
   <si>
-    <t xml:space="preserve">Emelda Waiya, Premila Lugstein, Isabella Nikodinovski: office roles on a production/technical agreement. Likely Clerks Private Sector Award [MA000002].</t>
+    <t xml:space="preserve">Emelda Waiya and Isabella Nikodinovski: office roles on a production/technical agreement. Likely Clerks Private Sector Award [MA000002]. Premila Lugstein does professional accounting work, so she is award free.</t>
   </si>
   <si>
     <t xml:space="preserve">5. Leave template / state problems</t>
@@ -136,7 +136,7 @@
     <t xml:space="preserve">Clerks Private Sector Award [MA000002]</t>
   </si>
   <si>
-    <t xml:space="preserve">Coverage summary. Likely award for office/admin staff (Emelda Waiya, Premila Lugstein, Isabella Nikodinovski).</t>
+    <t xml:space="preserve">Coverage summary. Likely award for office/admin staff (Emelda Waiya, Isabella Nikodinovski).</t>
   </si>
   <si>
     <t xml:space="preserve">https://fairwork.gov.au/awards-and-agreements/awards/award-summary/ma000002-summary</t>
@@ -973,10 +973,10 @@
     <t xml:space="preserve">Accountant (OFFICE / ADMIN) on a Production &amp; Support Level 5 agreement. Could be Clerks award or award-free depending on duties and pay. Check.</t>
   </si>
   <si>
-    <t xml:space="preserve">CHECK: Clerks Private Sector Award 2020 [MA000002] or award free</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clerks award if the work is accounts clerk work. Award free if it is professional accounting work. Contract and duties decide.</t>
+    <t xml:space="preserve">Award free (professional accounting work)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed professional accounting duties. Currently on Production &amp; Support Staff Level 5 agreement in EH. National Employment Standards and minimum wage still apply.</t>
   </si>
   <si>
     <t xml:space="preserve">Raigardas</t>
@@ -7580,9 +7580,7 @@
       <c r="X63" s="22"/>
       <c r="Y63" s="22"/>
       <c r="Z63" s="22"/>
-      <c r="AA63" s="22" t="s">
-        <v>167</v>
-      </c>
+      <c r="AA63" s="22"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="17" t="s">

</xml_diff>

<commit_message>
Register: casual loading confirmed from pay run 8, four casuals below the Live Performance Award base rate
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RNuMJNauftwNAHeyi1xsmD
</commit_message>
<xml_diff>
--- a/awards/CTS_Payroll_Setup_Register_21102026.xlsx
+++ b/awards/CTS_Payroll_Setup_Register_21102026.xlsx
@@ -34,19 +34,19 @@
     <t xml:space="preserve">Source: EH Employee Details Report, generated 21/10/2026, 79 currently employed staff.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. CHECK THIS FIRST: casual loading</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Casual rates are at or below permanent rates at the same level (e.g. casual Level 4 mostly $30.00 vs permanent Level 4 $30.05 to $33.70).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Either (a) the 25% casual loading is set on the "Casual Ordinary Hours" pay category in EH and added on top, or (b) casuals are not getting their loading.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check: Payroll Settings &gt; Pay Categories &gt; Casual Ordinary Hours &gt; look for a loading %. If there is no loading, this is the biggest risk in the file.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">See column Q on the Register tab.</t>
+    <t xml:space="preserve">1. Casual loading: CHECKED 21/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EH adds the 25% casual loading on top of the rate in column G. Pay run 8 (fortnight ending 16/10/2026): Chris Doherty $32.80 paid at $41.00, Elena Almaraz Ruiz $31.00 paid at $38.75. So column G is the base rate before loading.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compare column G to the Live Performance Award base rate, not the casual rate. Base rates from 1 July 2026: Level 3 $28.89, Level 4 $29.45, Level 5 $30.37, Level 6 $31.30.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Four casuals are below the award base rate: Emmett Todd, Jeffrey Kempin, Morgan Palmer, Zed Norrie. See column U on the Register tab.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Column Q (below lowest permanent) compares to permanent rates, not the award. Use column U for the award check.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Employment type does not match setup</t>
@@ -640,7 +640,7 @@
     <t xml:space="preserve">Casual SA</t>
   </si>
   <si>
-    <t xml:space="preserve">Casual Level 4 at $27.17, lower than other casual Level 4s ($30.00) and below every permanent Level 4. Check against agreement/award minimum for Level 4.</t>
+    <t xml:space="preserve">BELOW AWARD. EH rate $27.17 is the base before the 25% loading. Live Performance Award Level 4 base is $29.45 from 1 July 2026. Change the EH rate to at least $29.45 and work out back pay from the first pay period on or after 1 July 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Gabriela</t>
@@ -772,7 +772,7 @@
     <t xml:space="preserve">PWC - MEL Tech [ONS]</t>
   </si>
   <si>
-    <t xml:space="preserve">Casual Level 4 at $28.12, lower than other casual Level 4s ($30.00) and below every permanent Level 4. Check against agreement/award minimum for Level 4.</t>
+    <t xml:space="preserve">BELOW AWARD. EH rate $28.12 is the base before the 25% loading. Live Performance Award Level 4 base is $29.45 from 1 July 2026. Change the EH rate to at least $29.45 and work out back pay from the first pay period on or after 1 July 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Jeremy</t>
@@ -937,7 +937,7 @@
     <t xml:space="preserve">PWC IT P/T BNE [ONS]</t>
   </si>
   <si>
-    <t xml:space="preserve">Casual Level 5 at $29.00, lowest casual Level 5 and lower than most casual Level 4s. Check classification and minimum rate.</t>
+    <t xml:space="preserve">BELOW AWARD. EH rate $29.00 is the base before the 25% loading. Live Performance Award Level 5 base is $30.37 from 1 July 2026. Change the EH rate to at least $30.37 and work out back pay from the first pay period on or after 1 July 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Nicholas</t>
@@ -7267,7 +7267,7 @@
         <v/>
       </c>
       <c r="T59" s="25" t="s">
-        <v>147</v>
+        <v>100</v>
       </c>
       <c r="U59" s="21" t="s">
         <v>303</v>
@@ -8969,7 +8969,7 @@
         <v/>
       </c>
       <c r="T80" s="25" t="s">
-        <v>147</v>
+        <v>100</v>
       </c>
       <c r="U80" s="21" t="s">
         <v>303</v>

</xml_diff>